<commit_message>
einfach sachen schön gemacht
</commit_message>
<xml_diff>
--- a/results/analysis/full_analysis_ready_deduped.xlsx
+++ b/results/analysis/full_analysis_ready_deduped.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SinaElBasiouni\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SinaElBasiouni\Documents\3_Semester\Thesis\data\class_conscious_organization_files\results\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EED455B-57D2-403A-8403-7C00A9FE9B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091E087A-54B2-485F-936A-C0DAEBDCF19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1958,6 +1958,7 @@
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="35" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="15" max="15" width="8.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="58" x14ac:dyDescent="0.35">

</xml_diff>